<commit_message>
updated naming in metric result file
</commit_message>
<xml_diff>
--- a/Results/Assessing evaluation Metrics.xlsx
+++ b/Results/Assessing evaluation Metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Semester 4\Masters Thesis New\1. New Report Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32394258-C096-4F2C-A191-B1B5D4B95B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFCBAB7-67AD-4A0D-8343-53E9BF3027A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="XGBoost - Metrics" sheetId="1" r:id="rId1"/>
@@ -68,9 +68,6 @@
     <t>Integrated Gradient Global</t>
   </si>
   <si>
-    <t>Model</t>
-  </si>
-  <si>
     <t>Faithfulness</t>
   </si>
   <si>
@@ -129,6 +126,9 @@
   </si>
   <si>
     <t>Not Feasible</t>
+  </si>
+  <si>
+    <t>Metric</t>
   </si>
 </sst>
 </file>
@@ -778,6 +778,9 @@
     <xf numFmtId="166" fontId="18" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -787,16 +790,13 @@
     <xf numFmtId="0" fontId="19" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="0" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -846,68 +846,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1233,23 +1172,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="24"/>
+      <c r="A1" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>0</v>
@@ -1275,7 +1214,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="5">
         <v>0.88919999999999999</v>
@@ -1284,7 +1223,7 @@
         <v>-6.1199999999999997E-2</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="5">
         <v>-1.2999999999999999E-3</v>
@@ -1301,7 +1240,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="5">
         <v>2.1399999999999999E-2</v>
@@ -1313,13 +1252,13 @@
         <v>0.13070000000000001</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1327,7 +1266,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="5">
         <v>1.7487999999999999</v>
@@ -1336,7 +1275,7 @@
         <v>0.36859999999999998</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F5" s="5">
         <v>1.2522</v>
@@ -1345,7 +1284,7 @@
         <v>0.41320000000000001</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -1353,7 +1292,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="5">
         <v>0.89219999999999999</v>
@@ -1365,13 +1304,13 @@
         <v>1.0759000000000001</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1401,23 +1340,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="24"/>
+      <c r="A1" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>0</v>
@@ -1443,7 +1382,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="5">
         <v>0.99399999999999999</v>
@@ -1469,7 +1408,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="5">
         <v>-0.68540000000000001</v>
@@ -1481,13 +1420,13 @@
         <v>-0.27110000000000001</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1495,7 +1434,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" s="5">
         <v>1.1102000000000001</v>
@@ -1504,7 +1443,7 @@
         <v>0.95189999999999997</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F5" s="5">
         <v>3.2000000000000002E-3</v>
@@ -1513,7 +1452,7 @@
         <v>0.8851</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -1521,7 +1460,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="5">
         <v>7.0677000000000003</v>
@@ -1533,13 +1472,13 @@
         <v>4.43</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1570,25 +1509,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
+      <c r="A1" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
     </row>
     <row r="2" spans="1:10" ht="42" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>9</v>
+      <c r="B2" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>0</v>
@@ -1620,7 +1559,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="5">
         <v>0.96160000000000001</v>
@@ -1652,7 +1591,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="5">
         <v>-0.2616</v>
@@ -1664,19 +1603,19 @@
         <v>-0.2069</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I4" s="5">
         <v>-0.28860000000000002</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -1684,16 +1623,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="27">
+        <v>10</v>
+      </c>
+      <c r="C5" s="22">
         <v>0</v>
       </c>
       <c r="D5" s="5">
         <v>6.3700000000000007E-2</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F5" s="5">
         <v>2.3E-3</v>
@@ -1702,7 +1641,7 @@
         <v>0.55320000000000003</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I5" s="5">
         <v>2.5999999999999999E-3</v>
@@ -1716,7 +1655,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="5">
         <v>2.3519999999999999</v>
@@ -1728,19 +1667,19 @@
         <v>11.2704</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I6" s="5">
         <v>3.9895258169896597E-5</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1764,25 +1703,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="A1" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1970,25 +1909,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="A1" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>24</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -2176,25 +2115,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="A1" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="17" t="s">
         <v>22</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>